<commit_message>
Handoff kit: add 'materials to send' ask + asset-intake tracker tab
Yael has more materials/assets to share. Add an 'Anything you've already got?'
section to the email (html/md/docx) listing the useful items, and a new
'Assets to gather' sheet in the tracker mapping each asset to where it lands on
the site (covers auto-drop into assets/covers/<slug>.jpg, ebook files → Payhip,
photo/bio → About, etc.) with a Received? dropdown.
</commit_message>
<xml_diff>
--- a/handoff/yaels-letters-tracker.xlsx
+++ b/handoff/yaels-letters-tracker.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Follow-ups" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Links &amp; Logins" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets to gather" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1369,4 +1370,349 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Asset</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Where it goes on the site</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Format / spec</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Received?</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>'Letters from the Hill' ebook file</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Uploaded to Payhip (sold + delivered)</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>PDF or EPUB</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>The actual book</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>'Before the Rooster' ebook file</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Uploaded to Payhip (sold + delivered)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>PDF or EPUB</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>'Letters from the Hill' cover art</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>assets/covers/letters-from-the-hill.jpg</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Portrait ~448x624px (2x), JPEG/WebP</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Drops in automatically</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>'Before the Rooster' cover art</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>assets/covers/before-the-rooster.jpg</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Portrait ~448x624px (2x), JPEG/WebP</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Drops in automatically</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Book blurb — Letters from the Hill</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Book page + Payhip description</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>A paragraph of text</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Book blurb — Before the Rooster</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Book page + Payhip description</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>A paragraph of text</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Prices (per book)</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>store.js + Payhip</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>e.g. $4.99</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Photo of Yael</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>About page</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Landscape or portrait, good res</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Short bio / 'about Yael'</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>About page</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>A few sentences</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Reader notes / endorsements</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Books or home (optional feature)</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Short quotes + names</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Logo / wordmark</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Site branding / favicon</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>PNG/SVG, transparent</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Facebook / contact links</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Footer links</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>URLs</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="D2:D13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No,Received,N/A"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>